<commit_message>
Add Schedule FA for Mohammad Waseem Individual and Joint
FY2026-27 YTD Activity Statements for U25039405 and U24577010; seed GOOG
FOP/Internal costs; Internal transfers excluded from taxable CG; report
FY2026-27 capital gains and dividends.

Co-authored-by: caakshay-ux <caakshay-ux@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Foreign_Assets_Schedule_FA_Tushar_Agrawal_AY2026-27.xlsx
+++ b/output/Foreign_Assets_Schedule_FA_Tushar_Agrawal_AY2026-27.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1025,45 +1025,55 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HKD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>0.12849</v>
+        <v>1.342</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>JPY</t>
+          <t>HKD</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0.0063827</v>
+        <v>0.12849</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SGD</t>
+          <t>JPY</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>0.7776049766718507</v>
+        <v>0.0063827</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>SGD</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
+        <v>0.7776049766718507</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Yellow/input cells on CG sheets: Sale/Cost FCY, Comm USD, FX rates. All P&amp;L columns are formulas.</t>
         </is>

</xml_diff>